<commit_message>
Configure 400 Selenium E2E test cases and set up only appium mobile test report workflow
</commit_message>
<xml_diff>
--- a/volunteersync/test/e2e/reports/appium_e2e_report.xlsx
+++ b/volunteersync/test/e2e/reports/appium_e2e_report.xlsx
@@ -20,7 +20,7 @@
     <t>Generated At</t>
   </si>
   <si>
-    <t>23/6/2026, 12:06:43 pm</t>
+    <t>23/7/2026, 9:38:29 am</t>
   </si>
   <si>
     <t>Suite</t>
@@ -142,7 +142,7 @@
     <t>Landing screen renders with hero text "VolunteerSync"</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:33.791Z</t>
+    <t>2026-07-23T04:08:20.449Z</t>
   </si>
   <si>
     <t>Mocked execution – no real device required</t>
@@ -165,7 +165,7 @@
     <t>"Get Started" button is visible and clickable</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:33.855Z</t>
+    <t>2026-07-23T04:08:20.510Z</t>
   </si>
   <si>
     <t>LND-APP-03</t>
@@ -184,7 +184,7 @@
     <t>VolunteerSync logo/brand is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:33.896Z</t>
+    <t>2026-07-23T04:08:20.538Z</t>
   </si>
   <si>
     <t>LND-APP-04</t>
@@ -201,7 +201,7 @@
     <t>Login screen loads with email and password fields</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:33.937Z</t>
+    <t>2026-07-23T04:08:20.566Z</t>
   </si>
   <si>
     <t>LND-APP-05</t>
@@ -218,7 +218,7 @@
     <t>Feature cards render correctly when scrolled</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:33.965Z</t>
+    <t>2026-07-23T04:08:20.595Z</t>
   </si>
   <si>
     <t>LND-APP-06</t>
@@ -237,7 +237,7 @@
     <t>Footer with copyright text is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:33.999Z</t>
+    <t>2026-07-23T04:08:20.631Z</t>
   </si>
   <si>
     <t>LND-APP-07</t>
@@ -257,7 +257,7 @@
     <t>Tagline reads "Empowering Volunteers, Building Communities"</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.026Z</t>
+    <t>2026-07-23T04:08:20.658Z</t>
   </si>
   <si>
     <t>LND-APP-08</t>
@@ -274,7 +274,7 @@
     <t>Register form with name/email/password fields is visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.062Z</t>
+    <t>2026-07-23T04:08:20.685Z</t>
   </si>
   <si>
     <t>LND-APP-09</t>
@@ -291,7 +291,7 @@
     <t>Hero elements fade in without visual glitches</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.094Z</t>
+    <t>2026-07-23T04:08:20.711Z</t>
   </si>
   <si>
     <t>LND-APP-10</t>
@@ -307,7 +307,7 @@
     <t>Nav has: Home, Features, About, Get Started</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.130Z</t>
+    <t>2026-07-23T04:08:20.747Z</t>
   </si>
   <si>
     <t>LOG-APP-01</t>
@@ -323,7 +323,7 @@
     <t>All Login form elements are visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.165Z</t>
+    <t>2026-07-23T04:08:20.776Z</t>
   </si>
   <si>
     <t>LOG-APP-02</t>
@@ -343,7 +343,7 @@
     <t>Email and password validation errors are shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.204Z</t>
+    <t>2026-07-23T04:08:20.801Z</t>
   </si>
   <si>
     <t>LOG-APP-03</t>
@@ -360,7 +360,7 @@
     <t>"Enter a valid email address" error is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.232Z</t>
+    <t>2026-07-23T04:08:20.829Z</t>
   </si>
   <si>
     <t>LOG-APP-04</t>
@@ -378,7 +378,7 @@
     <t>"Password must be at least 6 characters" error is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.265Z</t>
+    <t>2026-07-23T04:08:20.857Z</t>
   </si>
   <si>
     <t>LOG-APP-05</t>
@@ -395,7 +395,7 @@
     <t>Forgot Password screen is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.303Z</t>
+    <t>2026-07-23T04:08:20.892Z</t>
   </si>
   <si>
     <t>LOG-APP-06</t>
@@ -412,7 +412,7 @@
     <t>Register screen loads correctly</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.338Z</t>
+    <t>2026-07-23T04:08:20.920Z</t>
   </si>
   <si>
     <t>LOG-APP-07</t>
@@ -433,7 +433,7 @@
     <t>Password toggle shows/hides password characters</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.396Z</t>
+    <t>2026-07-23T04:08:20.961Z</t>
   </si>
   <si>
     <t>LOG-APP-08</t>
@@ -450,7 +450,7 @@
     <t>User is logged in and Dashboard loads</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.436Z</t>
+    <t>2026-07-23T04:08:20.992Z</t>
   </si>
   <si>
     <t>LOG-APP-09</t>
@@ -467,7 +467,7 @@
     <t>"Invalid credentials" snackbar is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.476Z</t>
+    <t>2026-07-23T04:08:21.031Z</t>
   </si>
   <si>
     <t>LOG-APP-10</t>
@@ -483,7 +483,7 @@
     <t>Background gradient is visible and matches design</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.516Z</t>
+    <t>2026-07-23T04:08:21.066Z</t>
   </si>
   <si>
     <t>LOG-APP-11</t>
@@ -504,7 +504,7 @@
     <t>Keyboard opens and text is entered correctly</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.547Z</t>
+    <t>2026-07-23T04:08:21.093Z</t>
   </si>
   <si>
     <t>LOG-APP-12</t>
@@ -521,7 +521,7 @@
     <t>Focus moves to password field</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.595Z</t>
+    <t>2026-07-23T04:08:21.123Z</t>
   </si>
   <si>
     <t>REG-APP-01</t>
@@ -537,7 +537,7 @@
     <t>All registration fields are visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.635Z</t>
+    <t>2026-07-23T04:08:21.149Z</t>
   </si>
   <si>
     <t>REG-APP-02</t>
@@ -551,7 +551,7 @@
     <t>All required field validation errors are shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.671Z</t>
+    <t>2026-07-23T04:08:21.177Z</t>
   </si>
   <si>
     <t>REG-APP-03</t>
@@ -568,7 +568,7 @@
     <t>"Enter a valid email" error is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.703Z</t>
+    <t>2026-07-23T04:08:21.204Z</t>
   </si>
   <si>
     <t>REG-APP-04</t>
@@ -586,7 +586,7 @@
     <t>"Passwords do not match" error is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.733Z</t>
+    <t>2026-07-23T04:08:21.227Z</t>
   </si>
   <si>
     <t>REG-APP-05</t>
@@ -603,7 +603,7 @@
     <t>User account created and redirected to Dashboard</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.773Z</t>
+    <t>2026-07-23T04:08:21.251Z</t>
   </si>
   <si>
     <t>REG-APP-06</t>
@@ -619,7 +619,7 @@
     <t>Password strength indicator shows "Weak"</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.810Z</t>
+    <t>2026-07-23T04:08:21.274Z</t>
   </si>
   <si>
     <t>REG-APP-07</t>
@@ -636,7 +636,7 @@
     <t>Login screen is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.852Z</t>
+    <t>2026-07-23T04:08:21.307Z</t>
   </si>
   <si>
     <t>REG-APP-08</t>
@@ -654,7 +654,7 @@
     <t>"Name is required" validation error appears</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.894Z</t>
+    <t>2026-07-23T04:08:21.340Z</t>
   </si>
   <si>
     <t>REG-APP-09</t>
@@ -671,7 +671,7 @@
     <t>Role dropdown opens and selection is saved</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.942Z</t>
+    <t>2026-07-23T04:08:21.373Z</t>
   </si>
   <si>
     <t>REG-APP-10</t>
@@ -688,7 +688,7 @@
     <t>Both password fields toggle visibility independently</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:34.992Z</t>
+    <t>2026-07-23T04:08:21.407Z</t>
   </si>
   <si>
     <t>FP-APP-01</t>
@@ -704,7 +704,7 @@
     <t>Forgot Password form is fully visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.039Z</t>
+    <t>2026-07-23T04:08:21.440Z</t>
   </si>
   <si>
     <t>FP-APP-02</t>
@@ -720,7 +720,7 @@
     <t>"Email is required" error is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.074Z</t>
+    <t>2026-07-23T04:08:21.463Z</t>
   </si>
   <si>
     <t>FP-APP-03</t>
@@ -737,7 +737,7 @@
     <t>Success message "Password reset email sent" is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.112Z</t>
+    <t>2026-07-23T04:08:21.513Z</t>
   </si>
   <si>
     <t>FP-APP-04</t>
@@ -754,7 +754,7 @@
     <t>User returns to Login screen</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.155Z</t>
+    <t>2026-07-23T04:08:21.555Z</t>
   </si>
   <si>
     <t>FP-APP-05</t>
@@ -765,7 +765,7 @@
 3. Assert error</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.209Z</t>
+    <t>2026-07-23T04:08:21.593Z</t>
   </si>
   <si>
     <t>DASH-APP-01</t>
@@ -782,7 +782,7 @@
     <t>Dashboard renders with title "Dashboard Overview"</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.259Z</t>
+    <t>2026-07-23T04:08:21.621Z</t>
   </si>
   <si>
     <t>Mocked execution</t>
@@ -801,7 +801,7 @@
     <t>Greeting "Good morning, [FirstName] 👋" is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.304Z</t>
+    <t>2026-07-23T04:08:21.656Z</t>
   </si>
   <si>
     <t>DASH-APP-03</t>
@@ -818,7 +818,7 @@
     <t>Shimmer loading boxes appear while data is fetching</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.345Z</t>
+    <t>2026-07-23T04:08:21.683Z</t>
   </si>
   <si>
     <t>DASH-APP-04</t>
@@ -835,7 +835,7 @@
     <t>Total Volunteers card shows numeric count</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.387Z</t>
+    <t>2026-07-23T04:08:21.718Z</t>
   </si>
   <si>
     <t>DASH-APP-05</t>
@@ -851,7 +851,7 @@
     <t>Active Events card displays count</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.436Z</t>
+    <t>2026-07-23T04:08:21.754Z</t>
   </si>
   <si>
     <t>DASH-APP-06</t>
@@ -867,7 +867,7 @@
     <t>Hours This Month card renders with value</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.483Z</t>
+    <t>2026-07-23T04:08:21.794Z</t>
   </si>
   <si>
     <t>DASH-APP-07</t>
@@ -882,7 +882,7 @@
     <t>Attendance Rate card shows percentage value</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.514Z</t>
+    <t>2026-07-23T04:08:21.824Z</t>
   </si>
   <si>
     <t>DASH-APP-08</t>
@@ -897,7 +897,7 @@
     <t>All 4 stat cards have distinct gradient backgrounds</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.546Z</t>
+    <t>2026-07-23T04:08:21.871Z</t>
   </si>
   <si>
     <t>DASH-APP-09</t>
@@ -914,7 +914,7 @@
     <t>AI Insights banner shows volunteer recommendation text</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.590Z</t>
+    <t>2026-07-23T04:08:21.920Z</t>
   </si>
   <si>
     <t>DASH-APP-10</t>
@@ -930,7 +930,7 @@
     <t>AI Chat screen is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.629Z</t>
+    <t>2026-07-23T04:08:21.961Z</t>
   </si>
   <si>
     <t>DASH-APP-11</t>
@@ -946,7 +946,7 @@
     <t>Volunteer Growth line chart renders with 9 months data</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.673Z</t>
+    <t>2026-07-23T04:08:22.003Z</t>
   </si>
   <si>
     <t>DASH-APP-12</t>
@@ -962,7 +962,7 @@
     <t>Category pie chart renders with slices</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.745Z</t>
+    <t>2026-07-23T04:08:22.045Z</t>
   </si>
   <si>
     <t>DASH-APP-13</t>
@@ -978,7 +978,7 @@
     <t>Weekly Attendance bar chart is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.798Z</t>
+    <t>2026-07-23T04:08:22.086Z</t>
   </si>
   <si>
     <t>DASH-APP-14</t>
@@ -995,7 +995,7 @@
     <t>Recent Activity section shows at least 1 activity item</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.850Z</t>
+    <t>2026-07-23T04:08:22.114Z</t>
   </si>
   <si>
     <t>DASH-APP-15</t>
@@ -1010,7 +1010,7 @@
     <t>Activity items have all 3 content elements</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.890Z</t>
+    <t>2026-07-23T04:08:22.150Z</t>
   </si>
   <si>
     <t>DASH-APP-16</t>
@@ -1026,7 +1026,7 @@
     <t>Bottom nav bar shows all 6 navigation tabs</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.937Z</t>
+    <t>2026-07-23T04:08:22.190Z</t>
   </si>
   <si>
     <t>DASH-APP-17</t>
@@ -1042,7 +1042,7 @@
     <t>Volunteers screen is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:35.985Z</t>
+    <t>2026-07-23T04:08:22.227Z</t>
   </si>
   <si>
     <t>DASH-APP-18</t>
@@ -1058,7 +1058,7 @@
     <t>Events screen is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.040Z</t>
+    <t>2026-07-23T04:08:22.267Z</t>
   </si>
   <si>
     <t>DASH-APP-19</t>
@@ -1074,7 +1074,7 @@
     <t>Attendance screen is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.088Z</t>
+    <t>2026-07-23T04:08:22.308Z</t>
   </si>
   <si>
     <t>DASH-APP-20</t>
@@ -1090,7 +1090,7 @@
     <t>Reports screen is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.136Z</t>
+    <t>2026-07-23T04:08:22.357Z</t>
   </si>
   <si>
     <t>VOL-APP-01</t>
@@ -1107,7 +1107,7 @@
     <t>Volunteers screen renders with title and subtitle</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.195Z</t>
+    <t>2026-07-23T04:08:22.399Z</t>
   </si>
   <si>
     <t>VOL-APP-02</t>
@@ -1124,7 +1124,7 @@
     <t>Volunteer list renders with cards showing name and role</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.239Z</t>
+    <t>2026-07-23T04:08:22.440Z</t>
   </si>
   <si>
     <t>VOL-APP-03</t>
@@ -1141,7 +1141,7 @@
     <t>Shimmer placeholders appear during loading</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.293Z</t>
+    <t>2026-07-23T04:08:22.489Z</t>
   </si>
   <si>
     <t>VOL-APP-04</t>
@@ -1158,7 +1158,7 @@
     <t>Volunteer list filters by typed name</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.348Z</t>
+    <t>2026-07-23T04:08:22.532Z</t>
   </si>
   <si>
     <t>VOL-APP-05</t>
@@ -1174,7 +1174,7 @@
     <t>"No volunteers found" empty state is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.400Z</t>
+    <t>2026-07-23T04:08:22.579Z</t>
   </si>
   <si>
     <t>VOL-APP-06</t>
@@ -1191,7 +1191,7 @@
     <t>Full volunteer list is restored after clearing search</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.454Z</t>
+    <t>2026-07-23T04:08:22.621Z</t>
   </si>
   <si>
     <t>VOL-APP-07</t>
@@ -1207,7 +1207,7 @@
     <t>Only active volunteers are displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.506Z</t>
+    <t>2026-07-23T04:08:22.670Z</t>
   </si>
   <si>
     <t>VOL-APP-08</t>
@@ -1223,7 +1223,7 @@
     <t>Only inactive volunteers are displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.559Z</t>
+    <t>2026-07-23T04:08:22.718Z</t>
   </si>
   <si>
     <t>VOL-APP-09</t>
@@ -1240,7 +1240,7 @@
     <t>All volunteers are shown when "All" filter is selected</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.608Z</t>
+    <t>2026-07-23T04:08:22.760Z</t>
   </si>
   <si>
     <t>VOL-APP-10</t>
@@ -1256,7 +1256,7 @@
     <t>Volunteer card contains avatar, name, role, and skills</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.659Z</t>
+    <t>2026-07-23T04:08:22.789Z</t>
   </si>
   <si>
     <t>VOL-APP-11</t>
@@ -1271,7 +1271,7 @@
     <t>Hours and events count are visible on each card</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.701Z</t>
+    <t>2026-07-23T04:08:22.843Z</t>
   </si>
   <si>
     <t>VOL-APP-12</t>
@@ -1287,7 +1287,7 @@
     <t>Status badges show correct colors per status</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.759Z</t>
+    <t>2026-07-23T04:08:22.892Z</t>
   </si>
   <si>
     <t>VOL-APP-13</t>
@@ -1303,7 +1303,7 @@
     <t>Add Volunteer dialog opens with all form fields</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.814Z</t>
+    <t>2026-07-23T04:08:22.954Z</t>
   </si>
   <si>
     <t>VOL-APP-14</t>
@@ -1320,7 +1320,7 @@
     <t>Required field validation errors are shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.869Z</t>
+    <t>2026-07-23T04:08:22.996Z</t>
   </si>
   <si>
     <t>VOL-APP-15</t>
@@ -1338,7 +1338,7 @@
     <t>New volunteer is added and "Volunteer added!" snackbar shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.914Z</t>
+    <t>2026-07-23T04:08:23.052Z</t>
   </si>
   <si>
     <t>VOL-APP-16</t>
@@ -1356,7 +1356,7 @@
     <t>Dialog closes without creating a new volunteer</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:36.959Z</t>
+    <t>2026-07-23T04:08:23.100Z</t>
   </si>
   <si>
     <t>VOL-APP-17</t>
@@ -1373,7 +1373,7 @@
     <t>Email validation error is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.014Z</t>
+    <t>2026-07-23T04:08:23.149Z</t>
   </si>
   <si>
     <t>VOL-APP-18</t>
@@ -1390,7 +1390,7 @@
     <t>Volunteer detail sheet opens with full information</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.064Z</t>
+    <t>2026-07-23T04:08:23.190Z</t>
   </si>
   <si>
     <t>VOL-APP-19</t>
@@ -1407,7 +1407,7 @@
     <t>Skills list and events count are shown in detail view</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.114Z</t>
+    <t>2026-07-23T04:08:23.232Z</t>
   </si>
   <si>
     <t>VOL-APP-20</t>
@@ -1424,7 +1424,7 @@
     <t>Bottom sheet dismisses on downward swipe</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.178Z</t>
+    <t>2026-07-23T04:08:23.275Z</t>
   </si>
   <si>
     <t>VOL-APP-21</t>
@@ -1441,7 +1441,7 @@
     <t>Pull-to-refresh triggers data reload</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.227Z</t>
+    <t>2026-07-23T04:08:23.329Z</t>
   </si>
   <si>
     <t>VOL-APP-22</t>
@@ -1456,7 +1456,7 @@
     <t>Total volunteer count is visible on screen</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.275Z</t>
+    <t>2026-07-23T04:08:23.378Z</t>
   </si>
   <si>
     <t>EVT-APP-01</t>
@@ -1473,7 +1473,7 @@
     <t>Events screen renders correctly with title</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.324Z</t>
+    <t>2026-07-23T04:08:23.435Z</t>
   </si>
   <si>
     <t>EVT-APP-02</t>
@@ -1490,7 +1490,7 @@
     <t>Event cards render with title, location, and date</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.386Z</t>
+    <t>2026-07-23T04:08:23.489Z</t>
   </si>
   <si>
     <t>EVT-APP-03</t>
@@ -1506,7 +1506,7 @@
     <t>Shimmer boxes appear while events are loading</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.443Z</t>
+    <t>2026-07-23T04:08:23.523Z</t>
   </si>
   <si>
     <t>EVT-APP-04</t>
@@ -1523,7 +1523,7 @@
     <t>Events are filtered by search query</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.498Z</t>
+    <t>2026-07-23T04:08:23.565Z</t>
   </si>
   <si>
     <t>EVT-APP-05</t>
@@ -1539,7 +1539,7 @@
     <t>"No events found" empty state is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.546Z</t>
+    <t>2026-07-23T04:08:23.614Z</t>
   </si>
   <si>
     <t>EVT-APP-06</t>
@@ -1555,7 +1555,7 @@
     <t>All events are listed when "All" filter is active</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.613Z</t>
+    <t>2026-07-23T04:08:23.657Z</t>
   </si>
   <si>
     <t>EVT-APP-07</t>
@@ -1572,7 +1572,7 @@
     <t>Only upcoming events are displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.663Z</t>
+    <t>2026-07-23T04:08:23.704Z</t>
   </si>
   <si>
     <t>EVT-APP-08</t>
@@ -1588,7 +1588,7 @@
     <t>Only completed events are displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.727Z</t>
+    <t>2026-07-23T04:08:23.753Z</t>
   </si>
   <si>
     <t>EVT-APP-09</t>
@@ -1604,7 +1604,7 @@
     <t>Only draft events are displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.778Z</t>
+    <t>2026-07-23T04:08:23.808Z</t>
   </si>
   <si>
     <t>EVT-APP-10</t>
@@ -1621,7 +1621,7 @@
     <t>Each event card shows title, category, and status badge</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.842Z</t>
+    <t>2026-07-23T04:08:23.864Z</t>
   </si>
   <si>
     <t>EVT-APP-11</t>
@@ -1637,7 +1637,7 @@
     <t>Location and date are shown on event cards</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.900Z</t>
+    <t>2026-07-23T04:08:23.919Z</t>
   </si>
   <si>
     <t>EVT-APP-12</t>
@@ -1653,7 +1653,7 @@
     <t>Fill rate progress bar and percentage are visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:37.944Z</t>
+    <t>2026-07-23T04:08:23.975Z</t>
   </si>
   <si>
     <t>EVT-APP-13</t>
@@ -1669,7 +1669,7 @@
     <t>Event list is scrollable without layout issues</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.004Z</t>
+    <t>2026-07-23T04:08:24.016Z</t>
   </si>
   <si>
     <t>EVT-APP-14</t>
@@ -1685,7 +1685,7 @@
     <t>New Event dialog opens with all form fields</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.056Z</t>
+    <t>2026-07-23T04:08:24.067Z</t>
   </si>
   <si>
     <t>EVT-APP-15</t>
@@ -1702,7 +1702,7 @@
     <t>"Required" validation error on empty required fields</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.110Z</t>
+    <t>2026-07-23T04:08:24.135Z</t>
   </si>
   <si>
     <t>EVT-APP-16</t>
@@ -1719,7 +1719,7 @@
     <t>Event is created and success snackbar appears</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.160Z</t>
+    <t>2026-07-23T04:08:24.176Z</t>
   </si>
   <si>
     <t>EVT-APP-17</t>
@@ -1736,7 +1736,7 @@
     <t>All 6 categories (Education, Food Security, Environment, Health, Housing, Digital) visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.220Z</t>
+    <t>2026-07-23T04:08:24.219Z</t>
   </si>
   <si>
     <t>EVT-APP-18</t>
@@ -1754,7 +1754,7 @@
     <t>Dialog closes without creating an event</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.286Z</t>
+    <t>2026-07-23T04:08:24.273Z</t>
   </si>
   <si>
     <t>EVT-APP-19</t>
@@ -1771,7 +1771,7 @@
     <t>Event detail bottom sheet opens with full details</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.344Z</t>
+    <t>2026-07-23T04:08:24.322Z</t>
   </si>
   <si>
     <t>EVT-APP-20</t>
@@ -1787,7 +1787,7 @@
     <t>All event metadata is shown in detail sheet</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.396Z</t>
+    <t>2026-07-23T04:08:24.371Z</t>
   </si>
   <si>
     <t>EVT-APP-21</t>
@@ -1803,7 +1803,7 @@
     <t>KPI cards for volunteers registered and attended are visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.458Z</t>
+    <t>2026-07-23T04:08:24.434Z</t>
   </si>
   <si>
     <t>EVT-APP-22</t>
@@ -1819,7 +1819,7 @@
     <t>Tag chips are displayed in event detail</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.506Z</t>
+    <t>2026-07-23T04:08:24.489Z</t>
   </si>
   <si>
     <t>EVT-APP-23</t>
@@ -1836,7 +1836,7 @@
     <t>Manage Volunteers button is functional and closes the sheet</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.556Z</t>
+    <t>2026-07-23T04:08:24.538Z</t>
   </si>
   <si>
     <t>EVT-APP-24</t>
@@ -1853,7 +1853,7 @@
     <t>Bottom sheet expands and collapses on drag</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.622Z</t>
+    <t>2026-07-23T04:08:24.593Z</t>
   </si>
   <si>
     <t>ATT-APP-01</t>
@@ -1870,7 +1870,7 @@
     <t>Attendance screen renders with correct title and subtitle</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.692Z</t>
+    <t>2026-07-23T04:08:24.649Z</t>
   </si>
   <si>
     <t>ATT-APP-02</t>
@@ -1886,7 +1886,7 @@
     <t>Shimmer loading boxes appear during data fetch</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.758Z</t>
+    <t>2026-07-23T04:08:24.690Z</t>
   </si>
   <si>
     <t>ATT-APP-03</t>
@@ -1902,7 +1902,7 @@
     <t>All 4 summary chips render with numeric/percentage values</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.821Z</t>
+    <t>2026-07-23T04:08:24.753Z</t>
   </si>
   <si>
     <t>ATT-APP-04</t>
@@ -1920,7 +1920,7 @@
     <t>Each summary chip has the correct color coding</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.881Z</t>
+    <t>2026-07-23T04:08:24.809Z</t>
   </si>
   <si>
     <t>ATT-APP-05</t>
@@ -1936,7 +1936,7 @@
     <t>Tab bar renders with both tabs, Recent Records active by default</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.935Z</t>
+    <t>2026-07-23T04:08:24.871Z</t>
   </si>
   <si>
     <t>ATT-APP-06</t>
@@ -1953,7 +1953,7 @@
     <t>"By Event" tab shows attendance grouped by events</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:38.983Z</t>
+    <t>2026-07-23T04:08:24.934Z</t>
   </si>
   <si>
     <t>ATT-APP-07</t>
@@ -1969,7 +1969,7 @@
     <t>Recent Records tab shows individual check-in entries</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.039Z</t>
+    <t>2026-07-23T04:08:24.996Z</t>
   </si>
   <si>
     <t>ATT-APP-08</t>
@@ -1985,7 +1985,7 @@
     <t>Records list shows volunteer name, event, status icon</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.089Z</t>
+    <t>2026-07-23T04:08:25.058Z</t>
   </si>
   <si>
     <t>ATT-APP-09</t>
@@ -2002,7 +2002,7 @@
     <t>Status icons match the attendance status correctly</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.161Z</t>
+    <t>2026-07-23T04:08:25.121Z</t>
   </si>
   <si>
     <t>ATT-APP-10</t>
@@ -2018,7 +2018,7 @@
     <t>Check-in time and hours logged are shown on records</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.221Z</t>
+    <t>2026-07-23T04:08:25.176Z</t>
   </si>
   <si>
     <t>ATT-APP-11</t>
@@ -2034,7 +2034,7 @@
     <t>Records filter by volunteer name search query</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.279Z</t>
+    <t>2026-07-23T04:08:25.239Z</t>
   </si>
   <si>
     <t>ATT-APP-12</t>
@@ -2050,7 +2050,7 @@
     <t>Records filter by event name search query</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.329Z</t>
+    <t>2026-07-23T04:08:25.302Z</t>
   </si>
   <si>
     <t>ATT-APP-13</t>
@@ -2066,7 +2066,7 @@
     <t>"No records yet" empty state is shown for no results</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.396Z</t>
+    <t>2026-07-23T04:08:25.358Z</t>
   </si>
   <si>
     <t>ATT-APP-14</t>
@@ -2082,7 +2082,7 @@
     <t>Only present attendance records are displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.468Z</t>
+    <t>2026-07-23T04:08:25.430Z</t>
   </si>
   <si>
     <t>ATT-APP-15</t>
@@ -2098,7 +2098,7 @@
     <t>Only late attendance records are displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.523Z</t>
+    <t>2026-07-23T04:08:25.471Z</t>
   </si>
   <si>
     <t>ATT-APP-16</t>
@@ -2114,7 +2114,7 @@
     <t>Only absent records are displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.574Z</t>
+    <t>2026-07-23T04:08:25.513Z</t>
   </si>
   <si>
     <t>ATT-APP-17</t>
@@ -2131,7 +2131,7 @@
     <t>All attendance records are shown on "All" filter</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.636Z</t>
+    <t>2026-07-23T04:08:25.558Z</t>
   </si>
   <si>
     <t>ATT-APP-18</t>
@@ -2147,7 +2147,7 @@
     <t>Check-In dialog opens with form fields</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.709Z</t>
+    <t>2026-07-23T04:08:25.609Z</t>
   </si>
   <si>
     <t>ATT-APP-19</t>
@@ -2165,7 +2165,7 @@
     <t>"[Name] checked in successfully!" snackbar is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.775Z</t>
+    <t>2026-07-23T04:08:25.662Z</t>
   </si>
   <si>
     <t>ATT-APP-20</t>
@@ -2182,7 +2182,7 @@
     <t>Check-in is blocked when name field is empty</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.850Z</t>
+    <t>2026-07-23T04:08:25.704Z</t>
   </si>
   <si>
     <t>ATT-APP-21</t>
@@ -2199,7 +2199,7 @@
     <t>Event dropdown shows all available events</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.928Z</t>
+    <t>2026-07-23T04:08:25.746Z</t>
   </si>
   <si>
     <t>ATT-APP-22</t>
@@ -2216,7 +2216,7 @@
     <t>Dialog closes on Cancel without performing check-in</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:39.991Z</t>
+    <t>2026-07-23T04:08:25.803Z</t>
   </si>
   <si>
     <t>ATT-APP-23</t>
@@ -2232,7 +2232,7 @@
     <t>Each past event shows title, date, attendance rate, and progress bar</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.039Z</t>
+    <t>2026-07-23T04:08:25.871Z</t>
   </si>
   <si>
     <t>ATT-APP-24</t>
@@ -2249,7 +2249,7 @@
     <t>Progress bar colors reflect attendance rate correctly</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.089Z</t>
+    <t>2026-07-23T04:08:25.926Z</t>
   </si>
   <si>
     <t>ATT-APP-25</t>
@@ -2265,7 +2265,7 @@
     <t>"No past events" empty state is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.167Z</t>
+    <t>2026-07-23T04:08:25.982Z</t>
   </si>
   <si>
     <t>REP-APP-01</t>
@@ -2281,7 +2281,7 @@
     <t>Reports screen loads and title is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.241Z</t>
+    <t>2026-07-23T04:08:26.053Z</t>
   </si>
   <si>
     <t>REP-APP-02</t>
@@ -2296,7 +2296,7 @@
     <t>All 4 KPI cards render with values</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.305Z</t>
+    <t>2026-07-23T04:08:26.114Z</t>
   </si>
   <si>
     <t>REP-APP-03</t>
@@ -2312,7 +2312,7 @@
     <t>Volunteer hours chart is displayed with data</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.369Z</t>
+    <t>2026-07-23T04:08:26.183Z</t>
   </si>
   <si>
     <t>REP-APP-04</t>
@@ -2327,7 +2327,7 @@
     <t>Attendance trend chart is visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.442Z</t>
+    <t>2026-07-23T04:08:26.253Z</t>
   </si>
   <si>
     <t>REP-APP-05</t>
@@ -2342,7 +2342,7 @@
     <t>Category chart is visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.508Z</t>
+    <t>2026-07-23T04:08:26.308Z</t>
   </si>
   <si>
     <t>REP-APP-06</t>
@@ -2359,7 +2359,7 @@
     <t>Report data reflects This Week range</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.580Z</t>
+    <t>2026-07-23T04:08:26.364Z</t>
   </si>
   <si>
     <t>REP-APP-07</t>
@@ -2375,7 +2375,7 @@
     <t>Report reflects This Month data</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.645Z</t>
+    <t>2026-07-23T04:08:26.421Z</t>
   </si>
   <si>
     <t>REP-APP-08</t>
@@ -2391,7 +2391,7 @@
     <t>Report reflects Last 3 Months data</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.716Z</t>
+    <t>2026-07-23T04:08:26.482Z</t>
   </si>
   <si>
     <t>REP-APP-09</t>
@@ -2407,7 +2407,7 @@
     <t>Report reflects This Year data</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.763Z</t>
+    <t>2026-07-23T04:08:26.551Z</t>
   </si>
   <si>
     <t>REP-APP-10</t>
@@ -2423,7 +2423,7 @@
     <t>Export dialog or share sheet is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.838Z</t>
+    <t>2026-07-23T04:08:26.600Z</t>
   </si>
   <si>
     <t>REP-APP-11</t>
@@ -2439,7 +2439,7 @@
     <t>Top volunteers list renders with names and hours</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.909Z</t>
+    <t>2026-07-23T04:08:26.655Z</t>
   </si>
   <si>
     <t>REP-APP-12</t>
@@ -2454,7 +2454,7 @@
     <t>Skills distribution chart renders correctly</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:40.970Z</t>
+    <t>2026-07-23T04:08:26.718Z</t>
   </si>
   <si>
     <t>REP-APP-13</t>
@@ -2470,7 +2470,7 @@
     <t>Shimmer placeholders appear during data fetch</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.032Z</t>
+    <t>2026-07-23T04:08:26.773Z</t>
   </si>
   <si>
     <t>REP-APP-14</t>
@@ -2487,7 +2487,7 @@
     <t>Reports data refreshes successfully</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.105Z</t>
+    <t>2026-07-23T04:08:26.836Z</t>
   </si>
   <si>
     <t>REP-APP-15</t>
@@ -2502,7 +2502,7 @@
     <t>All KPI values are numeric and greater than zero</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.171Z</t>
+    <t>2026-07-23T04:08:26.899Z</t>
   </si>
   <si>
     <t>SET-APP-01</t>
@@ -2519,7 +2519,7 @@
     <t>Settings screen renders with title and subtitle</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.238Z</t>
+    <t>2026-07-23T04:08:26.970Z</t>
   </si>
   <si>
     <t>SET-APP-02</t>
@@ -2535,7 +2535,7 @@
     <t>Profile card shows all user information</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.311Z</t>
+    <t>2026-07-23T04:08:27.044Z</t>
   </si>
   <si>
     <t>SET-APP-03</t>
@@ -2552,7 +2552,7 @@
     <t>All 3 profile info rows are displayed with values</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.381Z</t>
+    <t>2026-07-23T04:08:27.107Z</t>
   </si>
   <si>
     <t>SET-APP-04</t>
@@ -2568,7 +2568,7 @@
     <t>Notifications section has all 4 toggle switches</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.449Z</t>
+    <t>2026-07-23T04:08:27.162Z</t>
   </si>
   <si>
     <t>SET-APP-05</t>
@@ -2586,7 +2586,7 @@
     <t>Email notifications toggle changes state on tap</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.513Z</t>
+    <t>2026-07-23T04:08:27.225Z</t>
   </si>
   <si>
     <t>SET-APP-06</t>
@@ -2602,7 +2602,7 @@
     <t>Push notifications toggle is functional</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.590Z</t>
+    <t>2026-07-23T04:08:27.271Z</t>
   </si>
   <si>
     <t>SET-APP-07</t>
@@ -2618,7 +2618,7 @@
     <t>AI insights toggle is functional</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.668Z</t>
+    <t>2026-07-23T04:08:27.315Z</t>
   </si>
   <si>
     <t>SET-APP-08</t>
@@ -2634,7 +2634,7 @@
     <t>Weekly digest toggle is functional</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.734Z</t>
+    <t>2026-07-23T04:08:27.380Z</t>
   </si>
   <si>
     <t>SET-APP-09</t>
@@ -2651,7 +2651,7 @@
     <t>Security section shows 2FA toggle and Change Password option</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.816Z</t>
+    <t>2026-07-23T04:08:27.435Z</t>
   </si>
   <si>
     <t>SET-APP-10</t>
@@ -2667,7 +2667,7 @@
     <t>2FA toggle is functional</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.890Z</t>
+    <t>2026-07-23T04:08:27.489Z</t>
   </si>
   <si>
     <t>SET-APP-11</t>
@@ -2683,7 +2683,7 @@
     <t>Password reset email is triggered and snackbar shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:41.969Z</t>
+    <t>2026-07-23T04:08:27.545Z</t>
   </si>
   <si>
     <t>SET-APP-12</t>
@@ -2700,7 +2700,7 @@
     <t>Language and Timezone dropdowns are visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.048Z</t>
+    <t>2026-07-23T04:08:27.616Z</t>
   </si>
   <si>
     <t>SET-APP-13</t>
@@ -2716,7 +2716,7 @@
     <t>Language dropdown shows all 4 supported languages</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.128Z</t>
+    <t>2026-07-23T04:08:27.685Z</t>
   </si>
   <si>
     <t>SET-APP-14</t>
@@ -2732,7 +2732,7 @@
     <t>Timezone dropdown shows all 4 US timezone options</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.185Z</t>
+    <t>2026-07-23T04:08:27.739Z</t>
   </si>
   <si>
     <t>SET-APP-15</t>
@@ -2749,7 +2749,7 @@
     <t>Language selection is reflected in the dropdown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.252Z</t>
+    <t>2026-07-23T04:08:27.811Z</t>
   </si>
   <si>
     <t>SET-APP-16</t>
@@ -2765,7 +2765,7 @@
     <t>About section shows all 4 info tiles</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.323Z</t>
+    <t>2026-07-23T04:08:27.879Z</t>
   </si>
   <si>
     <t>SET-APP-17</t>
@@ -2780,7 +2780,7 @@
     <t>App version is displayed as "1.0.0"</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.400Z</t>
+    <t>2026-07-23T04:08:27.949Z</t>
   </si>
   <si>
     <t>SET-APP-18</t>
@@ -2796,7 +2796,7 @@
     <t>"Coming soon!" snackbar is shown</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.460Z</t>
+    <t>2026-07-23T04:08:28.012Z</t>
   </si>
   <si>
     <t>SET-APP-19</t>
@@ -2809,7 +2809,7 @@
 2. Assert snackbar appears</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.518Z</t>
+    <t>2026-07-23T04:08:28.086Z</t>
   </si>
   <si>
     <t>SET-APP-20</t>
@@ -2825,7 +2825,7 @@
     <t>Snackbar shows "Contact: support@volunteersync.io"</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.585Z</t>
+    <t>2026-07-23T04:08:28.149Z</t>
   </si>
   <si>
     <t>SET-APP-21</t>
@@ -2838,7 +2838,7 @@
 2. Assert "Sign Out" outlined button visible</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.651Z</t>
+    <t>2026-07-23T04:08:28.204Z</t>
   </si>
   <si>
     <t>SET-APP-22</t>
@@ -2855,7 +2855,7 @@
     <t>User is signed out and Login screen is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.718Z</t>
+    <t>2026-07-23T04:08:28.274Z</t>
   </si>
   <si>
     <t>SET-APP-23</t>
@@ -2871,7 +2871,7 @@
     <t>Footer attribution text is displayed at bottom of Settings</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.792Z</t>
+    <t>2026-07-23T04:08:28.343Z</t>
   </si>
   <si>
     <t>AI-APP-01</t>
@@ -2887,7 +2887,7 @@
     <t>AI Chat screen loads with correct header</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.849Z</t>
+    <t>2026-07-23T04:08:28.398Z</t>
   </si>
   <si>
     <t>AI-APP-02</t>
@@ -2903,7 +2903,7 @@
     <t>Volt AI welcome message is displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.900Z</t>
+    <t>2026-07-23T04:08:28.468Z</t>
   </si>
   <si>
     <t>AI-APP-03</t>
@@ -2919,7 +2919,7 @@
     <t>Message input field is visible with placeholder text</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:42.965Z</t>
+    <t>2026-07-23T04:08:28.531Z</t>
   </si>
   <si>
     <t>AI-APP-04</t>
@@ -2936,7 +2936,7 @@
     <t>Typed text appears in the input field</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.026Z</t>
+    <t>2026-07-23T04:08:28.586Z</t>
   </si>
   <si>
     <t>AI-APP-05</t>
@@ -2953,7 +2953,7 @@
     <t>User message is sent and appears in chat as user bubble</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.097Z</t>
+    <t>2026-07-23T04:08:28.641Z</t>
   </si>
   <si>
     <t>AI-APP-06</t>
@@ -2970,7 +2970,7 @@
     <t>AI response is received and displayed</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.166Z</t>
+    <t>2026-07-23T04:08:28.697Z</t>
   </si>
   <si>
     <t>AI-APP-07</t>
@@ -2987,7 +2987,7 @@
     <t>User and AI messages have visually distinct bubble styles</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.230Z</t>
+    <t>2026-07-23T04:08:28.753Z</t>
   </si>
   <si>
     <t>AI-APP-08</t>
@@ -3003,7 +3003,7 @@
     <t>Loading indicator appears while AI generates response</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.303Z</t>
+    <t>2026-07-23T04:08:28.836Z</t>
   </si>
   <si>
     <t>AI-APP-09</t>
@@ -3020,7 +3020,7 @@
     <t>Input field is cleared after sending</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.368Z</t>
+    <t>2026-07-23T04:08:28.920Z</t>
   </si>
   <si>
     <t>AI-APP-10</t>
@@ -3036,7 +3036,7 @@
     <t>Chat auto-scrolls to the latest message</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.432Z</t>
+    <t>2026-07-23T04:08:28.975Z</t>
   </si>
   <si>
     <t>AI-APP-11</t>
@@ -3053,7 +3053,7 @@
     <t>Quick prompt chips are functional</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.491Z</t>
+    <t>2026-07-23T04:08:29.058Z</t>
   </si>
   <si>
     <t>AI-APP-12</t>
@@ -3071,7 +3071,7 @@
     <t>Chat messages are preserved when revisiting the screen</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.563Z</t>
+    <t>2026-07-23T04:08:29.138Z</t>
   </si>
   <si>
     <t>AI-APP-13</t>
@@ -3088,7 +3088,7 @@
     <t>Chat history is cleared after reset</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.636Z</t>
+    <t>2026-07-23T04:08:29.218Z</t>
   </si>
   <si>
     <t>AI-APP-14</t>
@@ -3105,7 +3105,7 @@
     <t>Empty message is not sent</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.699Z</t>
+    <t>2026-07-23T04:08:29.281Z</t>
   </si>
   <si>
     <t>AI-APP-15</t>
@@ -3122,7 +3122,7 @@
     <t>Back navigation returns to previous screen</t>
   </si>
   <si>
-    <t>2026-06-23T06:36:43.769Z</t>
+    <t>2026-07-23T04:08:29.364Z</t>
   </si>
 </sst>
 </file>
@@ -3970,7 +3970,7 @@
         <v>6</v>
       </c>
       <c r="J2" s="4">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>42</v>
@@ -4008,7 +4008,7 @@
         <v>6</v>
       </c>
       <c r="J3" s="4">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>49</v>
@@ -4046,7 +4046,7 @@
         <v>6</v>
       </c>
       <c r="J4" s="4">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>55</v>
@@ -4084,7 +4084,7 @@
         <v>6</v>
       </c>
       <c r="J5" s="4">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>60</v>
@@ -4122,7 +4122,7 @@
         <v>6</v>
       </c>
       <c r="J6" s="4">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>65</v>
@@ -4160,7 +4160,7 @@
         <v>6</v>
       </c>
       <c r="J7" s="4">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>71</v>
@@ -4198,7 +4198,7 @@
         <v>6</v>
       </c>
       <c r="J8" s="4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>77</v>
@@ -4274,7 +4274,7 @@
         <v>6</v>
       </c>
       <c r="J10" s="4">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>87</v>
@@ -4350,7 +4350,7 @@
         <v>6</v>
       </c>
       <c r="J12" s="4">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K12" s="4" t="s">
         <v>97</v>
@@ -4388,7 +4388,7 @@
         <v>6</v>
       </c>
       <c r="J13" s="4">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>103</v>
@@ -4426,7 +4426,7 @@
         <v>6</v>
       </c>
       <c r="J14" s="4">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>108</v>
@@ -4464,7 +4464,7 @@
         <v>6</v>
       </c>
       <c r="J15" s="4">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="K15" s="4" t="s">
         <v>113</v>
@@ -4502,7 +4502,7 @@
         <v>6</v>
       </c>
       <c r="J16" s="4">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K16" s="4" t="s">
         <v>118</v>
@@ -4540,7 +4540,7 @@
         <v>6</v>
       </c>
       <c r="J17" s="4">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K17" s="4" t="s">
         <v>123</v>
@@ -4578,7 +4578,7 @@
         <v>6</v>
       </c>
       <c r="J18" s="4">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="K18" s="4" t="s">
         <v>129</v>
@@ -4616,7 +4616,7 @@
         <v>6</v>
       </c>
       <c r="J19" s="4">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="K19" s="4" t="s">
         <v>134</v>
@@ -4654,7 +4654,7 @@
         <v>6</v>
       </c>
       <c r="J20" s="4">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K20" s="4" t="s">
         <v>139</v>
@@ -4692,7 +4692,7 @@
         <v>6</v>
       </c>
       <c r="J21" s="4">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="K21" s="4" t="s">
         <v>144</v>
@@ -4730,7 +4730,7 @@
         <v>6</v>
       </c>
       <c r="J22" s="4">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K22" s="4" t="s">
         <v>150</v>
@@ -4768,7 +4768,7 @@
         <v>6</v>
       </c>
       <c r="J23" s="4">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="K23" s="4" t="s">
         <v>155</v>
@@ -4806,7 +4806,7 @@
         <v>6</v>
       </c>
       <c r="J24" s="4">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="K24" s="4" t="s">
         <v>160</v>
@@ -4844,7 +4844,7 @@
         <v>6</v>
       </c>
       <c r="J25" s="4">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="K25" s="4" t="s">
         <v>164</v>
@@ -4882,7 +4882,7 @@
         <v>6</v>
       </c>
       <c r="J26" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K26" s="4" t="s">
         <v>169</v>
@@ -4920,7 +4920,7 @@
         <v>6</v>
       </c>
       <c r="J27" s="4">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K27" s="4" t="s">
         <v>174</v>
@@ -4958,7 +4958,7 @@
         <v>6</v>
       </c>
       <c r="J28" s="4">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K28" s="4" t="s">
         <v>179</v>
@@ -4996,7 +4996,7 @@
         <v>6</v>
       </c>
       <c r="J29" s="4">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="K29" s="4" t="s">
         <v>184</v>
@@ -5034,7 +5034,7 @@
         <v>6</v>
       </c>
       <c r="J30" s="4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K30" s="4" t="s">
         <v>189</v>
@@ -5072,7 +5072,7 @@
         <v>6</v>
       </c>
       <c r="J31" s="4">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="K31" s="4" t="s">
         <v>194</v>
@@ -5110,7 +5110,7 @@
         <v>6</v>
       </c>
       <c r="J32" s="4">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="K32" s="4" t="s">
         <v>199</v>
@@ -5148,7 +5148,7 @@
         <v>6</v>
       </c>
       <c r="J33" s="4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="K33" s="4" t="s">
         <v>204</v>
@@ -5186,7 +5186,7 @@
         <v>6</v>
       </c>
       <c r="J34" s="4">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="K34" s="4" t="s">
         <v>209</v>
@@ -5224,7 +5224,7 @@
         <v>6</v>
       </c>
       <c r="J35" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K35" s="4" t="s">
         <v>214</v>
@@ -5262,7 +5262,7 @@
         <v>6</v>
       </c>
       <c r="J36" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K36" s="4" t="s">
         <v>219</v>
@@ -5300,7 +5300,7 @@
         <v>6</v>
       </c>
       <c r="J37" s="4">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="K37" s="4" t="s">
         <v>224</v>
@@ -5338,7 +5338,7 @@
         <v>6</v>
       </c>
       <c r="J38" s="4">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="K38" s="4" t="s">
         <v>227</v>
@@ -5376,7 +5376,7 @@
         <v>6</v>
       </c>
       <c r="J39" s="4">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="K39" s="4" t="s">
         <v>232</v>
@@ -5414,7 +5414,7 @@
         <v>6</v>
       </c>
       <c r="J40" s="4">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K40" s="4" t="s">
         <v>238</v>
@@ -5490,7 +5490,7 @@
         <v>6</v>
       </c>
       <c r="J42" s="4">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K42" s="4" t="s">
         <v>248</v>
@@ -5528,7 +5528,7 @@
         <v>6</v>
       </c>
       <c r="J43" s="4">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="K43" s="4" t="s">
         <v>253</v>
@@ -5604,7 +5604,7 @@
         <v>6</v>
       </c>
       <c r="J45" s="4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K45" s="4" t="s">
         <v>263</v>
@@ -5642,7 +5642,7 @@
         <v>6</v>
       </c>
       <c r="J46" s="4">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="K46" s="4" t="s">
         <v>268</v>
@@ -5680,7 +5680,7 @@
         <v>6</v>
       </c>
       <c r="J47" s="4">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K47" s="4" t="s">
         <v>273</v>
@@ -5718,7 +5718,7 @@
         <v>6</v>
       </c>
       <c r="J48" s="4">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="K48" s="4" t="s">
         <v>278</v>
@@ -5756,7 +5756,7 @@
         <v>6</v>
       </c>
       <c r="J49" s="4">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="K49" s="4" t="s">
         <v>283</v>
@@ -5794,7 +5794,7 @@
         <v>6</v>
       </c>
       <c r="J50" s="4">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="K50" s="4" t="s">
         <v>288</v>
@@ -5832,7 +5832,7 @@
         <v>6</v>
       </c>
       <c r="J51" s="4">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="K51" s="4" t="s">
         <v>293</v>
@@ -5870,7 +5870,7 @@
         <v>6</v>
       </c>
       <c r="J52" s="4">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="K52" s="4" t="s">
         <v>298</v>
@@ -5908,7 +5908,7 @@
         <v>6</v>
       </c>
       <c r="J53" s="4">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K53" s="4" t="s">
         <v>303</v>
@@ -5946,7 +5946,7 @@
         <v>6</v>
       </c>
       <c r="J54" s="4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K54" s="4" t="s">
         <v>308</v>
@@ -5984,7 +5984,7 @@
         <v>6</v>
       </c>
       <c r="J55" s="4">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="K55" s="4" t="s">
         <v>313</v>
@@ -6022,7 +6022,7 @@
         <v>6</v>
       </c>
       <c r="J56" s="4">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K56" s="4" t="s">
         <v>318</v>
@@ -6060,7 +6060,7 @@
         <v>6</v>
       </c>
       <c r="J57" s="4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K57" s="4" t="s">
         <v>323</v>
@@ -6098,7 +6098,7 @@
         <v>6</v>
       </c>
       <c r="J58" s="4">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="K58" s="4" t="s">
         <v>328</v>
@@ -6136,7 +6136,7 @@
         <v>6</v>
       </c>
       <c r="J59" s="4">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="K59" s="4" t="s">
         <v>333</v>
@@ -6174,7 +6174,7 @@
         <v>6</v>
       </c>
       <c r="J60" s="4">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="K60" s="4" t="s">
         <v>338</v>
@@ -6212,7 +6212,7 @@
         <v>6</v>
       </c>
       <c r="J61" s="4">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K61" s="4" t="s">
         <v>343</v>
@@ -6250,7 +6250,7 @@
         <v>6</v>
       </c>
       <c r="J62" s="4">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="K62" s="4" t="s">
         <v>348</v>
@@ -6288,7 +6288,7 @@
         <v>6</v>
       </c>
       <c r="J63" s="4">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="K63" s="4" t="s">
         <v>353</v>
@@ -6326,7 +6326,7 @@
         <v>6</v>
       </c>
       <c r="J64" s="4">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="K64" s="4" t="s">
         <v>358</v>
@@ -6364,7 +6364,7 @@
         <v>6</v>
       </c>
       <c r="J65" s="4">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K65" s="4" t="s">
         <v>363</v>
@@ -6402,7 +6402,7 @@
         <v>6</v>
       </c>
       <c r="J66" s="4">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K66" s="4" t="s">
         <v>368</v>
@@ -6440,7 +6440,7 @@
         <v>6</v>
       </c>
       <c r="J67" s="4">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K67" s="4" t="s">
         <v>373</v>
@@ -6478,7 +6478,7 @@
         <v>6</v>
       </c>
       <c r="J68" s="4">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="K68" s="4" t="s">
         <v>378</v>
@@ -6516,7 +6516,7 @@
         <v>6</v>
       </c>
       <c r="J69" s="4">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="K69" s="4" t="s">
         <v>383</v>
@@ -6554,7 +6554,7 @@
         <v>6</v>
       </c>
       <c r="J70" s="4">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="K70" s="4" t="s">
         <v>388</v>
@@ -6630,7 +6630,7 @@
         <v>6</v>
       </c>
       <c r="J72" s="4">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="K72" s="4" t="s">
         <v>398</v>
@@ -6668,7 +6668,7 @@
         <v>6</v>
       </c>
       <c r="J73" s="4">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="K73" s="4" t="s">
         <v>403</v>
@@ -6706,7 +6706,7 @@
         <v>6</v>
       </c>
       <c r="J74" s="4">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K74" s="4" t="s">
         <v>408</v>
@@ -6744,7 +6744,7 @@
         <v>6</v>
       </c>
       <c r="J75" s="4">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="K75" s="4" t="s">
         <v>413</v>
@@ -6782,7 +6782,7 @@
         <v>6</v>
       </c>
       <c r="J76" s="4">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="K76" s="4" t="s">
         <v>418</v>
@@ -6820,7 +6820,7 @@
         <v>6</v>
       </c>
       <c r="J77" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="K77" s="4" t="s">
         <v>423</v>
@@ -6858,7 +6858,7 @@
         <v>6</v>
       </c>
       <c r="J78" s="4">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="K78" s="4" t="s">
         <v>428</v>
@@ -6896,7 +6896,7 @@
         <v>6</v>
       </c>
       <c r="J79" s="4">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="K79" s="4" t="s">
         <v>433</v>
@@ -6934,7 +6934,7 @@
         <v>6</v>
       </c>
       <c r="J80" s="4">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="K80" s="4" t="s">
         <v>438</v>
@@ -6972,7 +6972,7 @@
         <v>6</v>
       </c>
       <c r="J81" s="4">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K81" s="4" t="s">
         <v>443</v>
@@ -7010,7 +7010,7 @@
         <v>6</v>
       </c>
       <c r="J82" s="4">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="K82" s="4" t="s">
         <v>448</v>
@@ -7048,7 +7048,7 @@
         <v>6</v>
       </c>
       <c r="J83" s="4">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="K83" s="4" t="s">
         <v>453</v>
@@ -7086,7 +7086,7 @@
         <v>6</v>
       </c>
       <c r="J84" s="4">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="K84" s="4" t="s">
         <v>458</v>
@@ -7124,7 +7124,7 @@
         <v>6</v>
       </c>
       <c r="J85" s="4">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="K85" s="4" t="s">
         <v>463</v>
@@ -7162,7 +7162,7 @@
         <v>6</v>
       </c>
       <c r="J86" s="4">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="K86" s="4" t="s">
         <v>468</v>
@@ -7200,7 +7200,7 @@
         <v>6</v>
       </c>
       <c r="J87" s="4">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K87" s="4" t="s">
         <v>473</v>
@@ -7238,7 +7238,7 @@
         <v>6</v>
       </c>
       <c r="J88" s="4">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="K88" s="4" t="s">
         <v>478</v>
@@ -7276,7 +7276,7 @@
         <v>6</v>
       </c>
       <c r="J89" s="4">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="K89" s="4" t="s">
         <v>483</v>
@@ -7314,7 +7314,7 @@
         <v>6</v>
       </c>
       <c r="J90" s="4">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="K90" s="4" t="s">
         <v>488</v>
@@ -7352,7 +7352,7 @@
         <v>6</v>
       </c>
       <c r="J91" s="4">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="K91" s="4" t="s">
         <v>493</v>
@@ -7390,7 +7390,7 @@
         <v>6</v>
       </c>
       <c r="J92" s="4">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="K92" s="4" t="s">
         <v>498</v>
@@ -7428,7 +7428,7 @@
         <v>6</v>
       </c>
       <c r="J93" s="4">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="K93" s="4" t="s">
         <v>503</v>
@@ -7504,7 +7504,7 @@
         <v>6</v>
       </c>
       <c r="J95" s="4">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="K95" s="4" t="s">
         <v>513</v>
@@ -7542,7 +7542,7 @@
         <v>6</v>
       </c>
       <c r="J96" s="4">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K96" s="4" t="s">
         <v>518</v>
@@ -7580,7 +7580,7 @@
         <v>6</v>
       </c>
       <c r="J97" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K97" s="4" t="s">
         <v>523</v>
@@ -7618,7 +7618,7 @@
         <v>6</v>
       </c>
       <c r="J98" s="4">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="K98" s="4" t="s">
         <v>528</v>
@@ -7656,7 +7656,7 @@
         <v>6</v>
       </c>
       <c r="J99" s="4">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="K99" s="4" t="s">
         <v>533</v>
@@ -7732,7 +7732,7 @@
         <v>6</v>
       </c>
       <c r="J101" s="4">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="K101" s="4" t="s">
         <v>543</v>
@@ -7770,7 +7770,7 @@
         <v>6</v>
       </c>
       <c r="J102" s="4">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K102" s="4" t="s">
         <v>548</v>
@@ -7808,7 +7808,7 @@
         <v>6</v>
       </c>
       <c r="J103" s="4">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K103" s="4" t="s">
         <v>553</v>
@@ -7846,7 +7846,7 @@
         <v>6</v>
       </c>
       <c r="J104" s="4">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="K104" s="4" t="s">
         <v>558</v>
@@ -7884,7 +7884,7 @@
         <v>6</v>
       </c>
       <c r="J105" s="4">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="K105" s="4" t="s">
         <v>563</v>
@@ -7922,7 +7922,7 @@
         <v>6</v>
       </c>
       <c r="J106" s="4">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="K106" s="4" t="s">
         <v>568</v>
@@ -7960,7 +7960,7 @@
         <v>6</v>
       </c>
       <c r="J107" s="4">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="K107" s="4" t="s">
         <v>573</v>
@@ -8036,7 +8036,7 @@
         <v>6</v>
       </c>
       <c r="J109" s="4">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="K109" s="4" t="s">
         <v>583</v>
@@ -8074,7 +8074,7 @@
         <v>6</v>
       </c>
       <c r="J110" s="4">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="K110" s="4" t="s">
         <v>588</v>
@@ -8112,7 +8112,7 @@
         <v>6</v>
       </c>
       <c r="J111" s="4">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="K111" s="4" t="s">
         <v>593</v>
@@ -8150,7 +8150,7 @@
         <v>6</v>
       </c>
       <c r="J112" s="4">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="K112" s="4" t="s">
         <v>598</v>
@@ -8188,7 +8188,7 @@
         <v>6</v>
       </c>
       <c r="J113" s="4">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K113" s="4" t="s">
         <v>603</v>
@@ -8226,7 +8226,7 @@
         <v>6</v>
       </c>
       <c r="J114" s="4">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="K114" s="4" t="s">
         <v>608</v>
@@ -8264,7 +8264,7 @@
         <v>6</v>
       </c>
       <c r="J115" s="4">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="K115" s="4" t="s">
         <v>613</v>
@@ -8302,7 +8302,7 @@
         <v>6</v>
       </c>
       <c r="J116" s="4">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K116" s="4" t="s">
         <v>618</v>
@@ -8340,7 +8340,7 @@
         <v>6</v>
       </c>
       <c r="J117" s="4">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="K117" s="4" t="s">
         <v>623</v>
@@ -8378,7 +8378,7 @@
         <v>6</v>
       </c>
       <c r="J118" s="4">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="K118" s="4" t="s">
         <v>628</v>
@@ -8416,7 +8416,7 @@
         <v>6</v>
       </c>
       <c r="J119" s="4">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="K119" s="4" t="s">
         <v>633</v>
@@ -8454,7 +8454,7 @@
         <v>6</v>
       </c>
       <c r="J120" s="4">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="K120" s="4" t="s">
         <v>638</v>
@@ -8492,7 +8492,7 @@
         <v>6</v>
       </c>
       <c r="J121" s="4">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="K121" s="4" t="s">
         <v>643</v>
@@ -8530,7 +8530,7 @@
         <v>6</v>
       </c>
       <c r="J122" s="4">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="K122" s="4" t="s">
         <v>648</v>
@@ -8606,7 +8606,7 @@
         <v>6</v>
       </c>
       <c r="J124" s="4">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="K124" s="4" t="s">
         <v>658</v>
@@ -8644,7 +8644,7 @@
         <v>6</v>
       </c>
       <c r="J125" s="4">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="K125" s="4" t="s">
         <v>663</v>
@@ -8720,7 +8720,7 @@
         <v>6</v>
       </c>
       <c r="J127" s="4">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="K127" s="4" t="s">
         <v>673</v>
@@ -8758,7 +8758,7 @@
         <v>6</v>
       </c>
       <c r="J128" s="4">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="K128" s="4" t="s">
         <v>678</v>
@@ -8796,7 +8796,7 @@
         <v>6</v>
       </c>
       <c r="J129" s="4">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="K129" s="4" t="s">
         <v>683</v>
@@ -8834,7 +8834,7 @@
         <v>6</v>
       </c>
       <c r="J130" s="4">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="K130" s="4" t="s">
         <v>688</v>
@@ -8910,7 +8910,7 @@
         <v>6</v>
       </c>
       <c r="J132" s="4">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="K132" s="4" t="s">
         <v>698</v>
@@ -8948,7 +8948,7 @@
         <v>6</v>
       </c>
       <c r="J133" s="4">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K133" s="4" t="s">
         <v>703</v>
@@ -8986,7 +8986,7 @@
         <v>6</v>
       </c>
       <c r="J134" s="4">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="K134" s="4" t="s">
         <v>708</v>
@@ -9024,7 +9024,7 @@
         <v>6</v>
       </c>
       <c r="J135" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K135" s="4" t="s">
         <v>713</v>
@@ -9062,7 +9062,7 @@
         <v>6</v>
       </c>
       <c r="J136" s="4">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K136" s="4" t="s">
         <v>718</v>
@@ -9100,7 +9100,7 @@
         <v>6</v>
       </c>
       <c r="J137" s="4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K137" s="4" t="s">
         <v>723</v>
@@ -9138,7 +9138,7 @@
         <v>6</v>
       </c>
       <c r="J138" s="4">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K138" s="4" t="s">
         <v>728</v>
@@ -9176,7 +9176,7 @@
         <v>6</v>
       </c>
       <c r="J139" s="4">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="K139" s="4" t="s">
         <v>733</v>
@@ -9214,7 +9214,7 @@
         <v>6</v>
       </c>
       <c r="J140" s="4">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="K140" s="4" t="s">
         <v>738</v>
@@ -9252,7 +9252,7 @@
         <v>6</v>
       </c>
       <c r="J141" s="4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="K141" s="4" t="s">
         <v>743</v>
@@ -9290,7 +9290,7 @@
         <v>6</v>
       </c>
       <c r="J142" s="4">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K142" s="4" t="s">
         <v>748</v>
@@ -9328,7 +9328,7 @@
         <v>6</v>
       </c>
       <c r="J143" s="4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K143" s="4" t="s">
         <v>753</v>
@@ -9366,7 +9366,7 @@
         <v>6</v>
       </c>
       <c r="J144" s="4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K144" s="4" t="s">
         <v>758</v>
@@ -9404,7 +9404,7 @@
         <v>6</v>
       </c>
       <c r="J145" s="4">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="K145" s="4" t="s">
         <v>763</v>
@@ -9442,7 +9442,7 @@
         <v>6</v>
       </c>
       <c r="J146" s="4">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="K146" s="4" t="s">
         <v>768</v>
@@ -9480,7 +9480,7 @@
         <v>6</v>
       </c>
       <c r="J147" s="4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="K147" s="4" t="s">
         <v>773</v>
@@ -9518,7 +9518,7 @@
         <v>6</v>
       </c>
       <c r="J148" s="4">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="K148" s="4" t="s">
         <v>778</v>
@@ -9556,7 +9556,7 @@
         <v>6</v>
       </c>
       <c r="J149" s="4">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="K149" s="4" t="s">
         <v>783</v>
@@ -9594,7 +9594,7 @@
         <v>6</v>
       </c>
       <c r="J150" s="4">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="K150" s="4" t="s">
         <v>788</v>
@@ -9632,7 +9632,7 @@
         <v>6</v>
       </c>
       <c r="J151" s="4">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="K151" s="4" t="s">
         <v>793</v>
@@ -9670,7 +9670,7 @@
         <v>6</v>
       </c>
       <c r="J152" s="4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K152" s="4" t="s">
         <v>798</v>
@@ -9708,7 +9708,7 @@
         <v>6</v>
       </c>
       <c r="J153" s="4">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="K153" s="4" t="s">
         <v>803</v>
@@ -9746,7 +9746,7 @@
         <v>6</v>
       </c>
       <c r="J154" s="4">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K154" s="4" t="s">
         <v>808</v>
@@ -9784,7 +9784,7 @@
         <v>6</v>
       </c>
       <c r="J155" s="4">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="K155" s="4" t="s">
         <v>813</v>
@@ -9860,7 +9860,7 @@
         <v>6</v>
       </c>
       <c r="J157" s="4">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="K157" s="4" t="s">
         <v>823</v>
@@ -9898,7 +9898,7 @@
         <v>6</v>
       </c>
       <c r="J158" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K158" s="4" t="s">
         <v>828</v>
@@ -9936,7 +9936,7 @@
         <v>6</v>
       </c>
       <c r="J159" s="4">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K159" s="4" t="s">
         <v>833</v>
@@ -9974,7 +9974,7 @@
         <v>6</v>
       </c>
       <c r="J160" s="4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="K160" s="4" t="s">
         <v>838</v>
@@ -10012,7 +10012,7 @@
         <v>6</v>
       </c>
       <c r="J161" s="4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K161" s="4" t="s">
         <v>843</v>
@@ -10050,7 +10050,7 @@
         <v>6</v>
       </c>
       <c r="J162" s="4">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K162" s="4" t="s">
         <v>848</v>
@@ -10088,7 +10088,7 @@
         <v>6</v>
       </c>
       <c r="J163" s="4">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K163" s="4" t="s">
         <v>852</v>
@@ -10126,7 +10126,7 @@
         <v>6</v>
       </c>
       <c r="J164" s="4">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K164" s="4" t="s">
         <v>857</v>
@@ -10164,7 +10164,7 @@
         <v>6</v>
       </c>
       <c r="J165" s="4">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="K165" s="4" t="s">
         <v>861</v>
@@ -10202,7 +10202,7 @@
         <v>6</v>
       </c>
       <c r="J166" s="4">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="K166" s="4" t="s">
         <v>866</v>
@@ -10278,7 +10278,7 @@
         <v>6</v>
       </c>
       <c r="J168" s="4">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K168" s="4" t="s">
         <v>876</v>
@@ -10354,7 +10354,7 @@
         <v>6</v>
       </c>
       <c r="J170" s="4">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K170" s="4" t="s">
         <v>886</v>
@@ -10392,7 +10392,7 @@
         <v>6</v>
       </c>
       <c r="J171" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K171" s="4" t="s">
         <v>891</v>
@@ -10430,7 +10430,7 @@
         <v>6</v>
       </c>
       <c r="J172" s="4">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K172" s="4" t="s">
         <v>896</v>
@@ -10468,7 +10468,7 @@
         <v>6</v>
       </c>
       <c r="J173" s="4">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="K173" s="4" t="s">
         <v>901</v>
@@ -10544,7 +10544,7 @@
         <v>6</v>
       </c>
       <c r="J175" s="4">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="K175" s="4" t="s">
         <v>911</v>
@@ -10582,7 +10582,7 @@
         <v>6</v>
       </c>
       <c r="J176" s="4">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="K176" s="4" t="s">
         <v>916</v>
@@ -10620,7 +10620,7 @@
         <v>6</v>
       </c>
       <c r="J177" s="4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K177" s="4" t="s">
         <v>921</v>
@@ -10658,7 +10658,7 @@
         <v>6</v>
       </c>
       <c r="J178" s="4">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="K178" s="4" t="s">
         <v>926</v>
@@ -10696,7 +10696,7 @@
         <v>6</v>
       </c>
       <c r="J179" s="4">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="K179" s="4" t="s">
         <v>931</v>
@@ -10734,7 +10734,7 @@
         <v>6</v>
       </c>
       <c r="J180" s="4">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="K180" s="4" t="s">
         <v>936</v>
@@ -10772,7 +10772,7 @@
         <v>6</v>
       </c>
       <c r="J181" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K181" s="4" t="s">
         <v>941</v>
@@ -10810,7 +10810,7 @@
         <v>6</v>
       </c>
       <c r="J182" s="4">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="K182" s="4" t="s">
         <v>946</v>

</xml_diff>